<commit_message>
Replace loading with explicit initial crystal states
</commit_message>
<xml_diff>
--- a/examples/fake-experimental-dataset.xlsx
+++ b/examples/fake-experimental-dataset.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="14">
   <si>
     <t>Exp_ID</t>
   </si>
@@ -34,9 +34,6 @@
   </si>
   <si>
     <t>Temperature</t>
-  </si>
-  <si>
-    <t>Loading</t>
   </si>
   <si>
     <t>Time</t>
@@ -54,7 +51,22 @@
     <t>PS_var</t>
   </si>
   <si>
+    <t>SeedMass</t>
+  </si>
+  <si>
+    <t>SeedD43</t>
+  </si>
+  <si>
+    <t>SeedDistribution</t>
+  </si>
+  <si>
+    <t>SeedSpread</t>
+  </si>
+  <si>
     <t>FAKE_SYS_A</t>
+  </si>
+  <si>
+    <t>lognormal</t>
   </si>
 </sst>
 </file>
@@ -406,10 +418,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CAF0E20E-E4D8-9B45-9C94-E89B574F109C}">
-  <dimension ref="A1:I57"/>
+  <dimension ref="A1:L57"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:12">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -437,13 +449,22 @@
       <c r="I1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" spans="1:9">
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C2">
         <v>11.85</v>
@@ -452,346 +473,454 @@
         <v>0.0</v>
       </c>
       <c r="E2">
-        <v>0.0</v>
+        <v>22.075068</v>
       </c>
       <c r="F2">
-        <v>22.075068</v>
+        <v>0.4356</v>
       </c>
       <c r="G2">
-        <v>0.4356</v>
+        <v>-1.0</v>
       </c>
       <c r="H2">
         <v>-1.0</v>
       </c>
       <c r="I2">
-        <v>-1.0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9">
+        <v>0.0</v>
+      </c>
+      <c r="J2">
+        <v>0.0</v>
+      </c>
+      <c r="K2" t="s">
+        <v>13</v>
+      </c>
+      <c r="L2">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12">
       <c r="A3">
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C3">
         <v>11.85</v>
       </c>
       <c r="D3">
-        <v>0.0</v>
+        <v>4.69</v>
       </c>
       <c r="E3">
-        <v>4.69</v>
+        <v>3.48283</v>
       </c>
       <c r="F3">
-        <v>3.48283</v>
+        <v>0.01094315</v>
       </c>
       <c r="G3">
-        <v>0.01094315</v>
+        <v>-1.0</v>
       </c>
       <c r="H3">
         <v>-1.0</v>
       </c>
       <c r="I3">
-        <v>-1.0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9">
+        <v>0.0</v>
+      </c>
+      <c r="J3">
+        <v>0.0</v>
+      </c>
+      <c r="K3" t="s">
+        <v>13</v>
+      </c>
+      <c r="L3">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12">
       <c r="A4">
         <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C4">
         <v>11.85</v>
       </c>
       <c r="D4">
-        <v>0.0</v>
+        <v>10.13</v>
       </c>
       <c r="E4">
-        <v>10.13</v>
+        <v>2.742553</v>
       </c>
       <c r="F4">
-        <v>2.742553</v>
+        <v>0.00661878</v>
       </c>
       <c r="G4">
-        <v>0.00661878</v>
+        <v>-1.0</v>
       </c>
       <c r="H4">
         <v>-1.0</v>
       </c>
       <c r="I4">
-        <v>-1.0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9">
+        <v>0.0</v>
+      </c>
+      <c r="J4">
+        <v>0.0</v>
+      </c>
+      <c r="K4" t="s">
+        <v>13</v>
+      </c>
+      <c r="L4">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12">
       <c r="A5">
         <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C5">
         <v>11.85</v>
       </c>
       <c r="D5">
-        <v>0.0</v>
+        <v>20.13</v>
       </c>
       <c r="E5">
-        <v>20.13</v>
+        <v>2.252195</v>
       </c>
       <c r="F5">
-        <v>2.252195</v>
+        <v>0.00461498</v>
       </c>
       <c r="G5">
-        <v>0.00461498</v>
+        <v>-1.0</v>
       </c>
       <c r="H5">
         <v>-1.0</v>
       </c>
       <c r="I5">
-        <v>-1.0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9">
+        <v>0.0</v>
+      </c>
+      <c r="J5">
+        <v>0.0</v>
+      </c>
+      <c r="K5" t="s">
+        <v>13</v>
+      </c>
+      <c r="L5">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12">
       <c r="A6">
         <v>1</v>
       </c>
       <c r="B6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C6">
         <v>11.85</v>
       </c>
       <c r="D6">
-        <v>0.0</v>
+        <v>30.43</v>
       </c>
       <c r="E6">
-        <v>30.43</v>
+        <v>2.061059</v>
       </c>
       <c r="F6">
-        <v>2.061059</v>
+        <v>0.00384691</v>
       </c>
       <c r="G6">
-        <v>0.00384691</v>
+        <v>-1.0</v>
       </c>
       <c r="H6">
         <v>-1.0</v>
       </c>
       <c r="I6">
-        <v>-1.0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9">
+        <v>0.0</v>
+      </c>
+      <c r="J6">
+        <v>0.0</v>
+      </c>
+      <c r="K6" t="s">
+        <v>13</v>
+      </c>
+      <c r="L6">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12">
       <c r="A7">
         <v>1</v>
       </c>
       <c r="B7" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C7">
         <v>11.85</v>
       </c>
       <c r="D7">
-        <v>0.0</v>
+        <v>60.1</v>
       </c>
       <c r="E7">
-        <v>60.1</v>
+        <v>1.858553</v>
       </c>
       <c r="F7">
-        <v>1.858553</v>
+        <v>0.00299827</v>
       </c>
       <c r="G7">
-        <v>0.00299827</v>
+        <v>-1.0</v>
       </c>
       <c r="H7">
         <v>-1.0</v>
       </c>
       <c r="I7">
-        <v>-1.0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9">
+        <v>0.0</v>
+      </c>
+      <c r="J7">
+        <v>0.0</v>
+      </c>
+      <c r="K7" t="s">
+        <v>13</v>
+      </c>
+      <c r="L7">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12">
       <c r="A8">
         <v>1</v>
       </c>
       <c r="B8" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C8">
         <v>11.85</v>
       </c>
       <c r="D8">
-        <v>0.0</v>
+        <v>89.65</v>
       </c>
       <c r="E8">
-        <v>89.65</v>
+        <v>1.616167</v>
       </c>
       <c r="F8">
-        <v>1.616167</v>
+        <v>0.0026585</v>
       </c>
       <c r="G8">
-        <v>0.0026585</v>
+        <v>-1.0</v>
       </c>
       <c r="H8">
         <v>-1.0</v>
       </c>
       <c r="I8">
-        <v>-1.0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9">
+        <v>0.0</v>
+      </c>
+      <c r="J8">
+        <v>0.0</v>
+      </c>
+      <c r="K8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L8">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12">
       <c r="A9">
         <v>1</v>
       </c>
       <c r="B9" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C9">
         <v>11.85</v>
       </c>
       <c r="D9">
-        <v>0.0</v>
+        <v>129.53</v>
       </c>
       <c r="E9">
-        <v>129.53</v>
+        <v>1.688958</v>
       </c>
       <c r="F9">
-        <v>1.688958</v>
+        <v>0.00241615</v>
       </c>
       <c r="G9">
-        <v>0.00241615</v>
+        <v>-1.0</v>
       </c>
       <c r="H9">
         <v>-1.0</v>
       </c>
       <c r="I9">
-        <v>-1.0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9">
+        <v>0.0</v>
+      </c>
+      <c r="J9">
+        <v>0.0</v>
+      </c>
+      <c r="K9" t="s">
+        <v>13</v>
+      </c>
+      <c r="L9">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12">
       <c r="A10">
         <v>1</v>
       </c>
       <c r="B10" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C10">
         <v>11.85</v>
       </c>
       <c r="D10">
-        <v>0.0</v>
+        <v>179.54</v>
       </c>
       <c r="E10">
-        <v>179.54</v>
+        <v>1.603835</v>
       </c>
       <c r="F10">
-        <v>1.603835</v>
+        <v>0.00224404</v>
       </c>
       <c r="G10">
-        <v>0.00224404</v>
+        <v>-1.0</v>
       </c>
       <c r="H10">
         <v>-1.0</v>
       </c>
       <c r="I10">
-        <v>-1.0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9">
+        <v>0.0</v>
+      </c>
+      <c r="J10">
+        <v>0.0</v>
+      </c>
+      <c r="K10" t="s">
+        <v>13</v>
+      </c>
+      <c r="L10">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12">
       <c r="A11">
         <v>1</v>
       </c>
       <c r="B11" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C11">
         <v>11.85</v>
       </c>
       <c r="D11">
-        <v>0.0</v>
+        <v>219.63</v>
       </c>
       <c r="E11">
-        <v>219.63</v>
+        <v>1.500094</v>
       </c>
       <c r="F11">
-        <v>1.500094</v>
+        <v>0.00215399</v>
       </c>
       <c r="G11">
-        <v>0.00215399</v>
+        <v>-1.0</v>
       </c>
       <c r="H11">
         <v>-1.0</v>
       </c>
       <c r="I11">
-        <v>-1.0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9">
+        <v>0.0</v>
+      </c>
+      <c r="J11">
+        <v>0.0</v>
+      </c>
+      <c r="K11" t="s">
+        <v>13</v>
+      </c>
+      <c r="L11">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12">
       <c r="A12">
         <v>1</v>
       </c>
       <c r="B12" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C12">
         <v>11.85</v>
       </c>
       <c r="D12">
-        <v>0.0</v>
+        <v>259.74</v>
       </c>
       <c r="E12">
-        <v>259.74</v>
+        <v>1.512917</v>
       </c>
       <c r="F12">
-        <v>1.512917</v>
+        <v>0.00208705</v>
       </c>
       <c r="G12">
-        <v>0.00208705</v>
+        <v>-1.0</v>
       </c>
       <c r="H12">
         <v>-1.0</v>
       </c>
       <c r="I12">
-        <v>-1.0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9">
+        <v>0.0</v>
+      </c>
+      <c r="J12">
+        <v>0.0</v>
+      </c>
+      <c r="K12" t="s">
+        <v>13</v>
+      </c>
+      <c r="L12">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12">
       <c r="A13">
         <v>1</v>
       </c>
       <c r="B13" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C13">
         <v>11.85</v>
       </c>
       <c r="D13">
-        <v>0.0</v>
+        <v>300.0</v>
       </c>
       <c r="E13">
-        <v>300.0</v>
+        <v>1.465559</v>
       </c>
       <c r="F13">
-        <v>1.465559</v>
+        <v>0.0020347</v>
       </c>
       <c r="G13">
-        <v>0.0020347</v>
+        <v>1.292773</v>
       </c>
       <c r="H13">
-        <v>1.292773</v>
+        <v>0.01036329</v>
       </c>
       <c r="I13">
-        <v>0.01036329</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9">
+        <v>0.0</v>
+      </c>
+      <c r="J13">
+        <v>0.0</v>
+      </c>
+      <c r="K13" t="s">
+        <v>13</v>
+      </c>
+      <c r="L13">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12">
       <c r="A14">
         <v>2</v>
       </c>
       <c r="B14" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C14">
         <v>14.85</v>
@@ -800,288 +929,378 @@
         <v>0.0</v>
       </c>
       <c r="E14">
-        <v>0.0</v>
+        <v>20.100007</v>
       </c>
       <c r="F14">
-        <v>20.100007</v>
+        <v>0.36</v>
       </c>
       <c r="G14">
-        <v>0.36</v>
+        <v>-1.0</v>
       </c>
       <c r="H14">
         <v>-1.0</v>
       </c>
       <c r="I14">
-        <v>-1.0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9">
+        <v>0.0</v>
+      </c>
+      <c r="J14">
+        <v>0.0</v>
+      </c>
+      <c r="K14" t="s">
+        <v>13</v>
+      </c>
+      <c r="L14">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12">
       <c r="A15">
         <v>2</v>
       </c>
       <c r="B15" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C15">
         <v>14.85</v>
       </c>
       <c r="D15">
-        <v>0.0</v>
+        <v>8.43</v>
       </c>
       <c r="E15">
-        <v>8.43</v>
+        <v>4.969409</v>
       </c>
       <c r="F15">
-        <v>4.969409</v>
+        <v>0.01910934</v>
       </c>
       <c r="G15">
-        <v>0.01910934</v>
+        <v>-1.0</v>
       </c>
       <c r="H15">
         <v>-1.0</v>
       </c>
       <c r="I15">
-        <v>-1.0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9">
+        <v>0.0</v>
+      </c>
+      <c r="J15">
+        <v>0.0</v>
+      </c>
+      <c r="K15" t="s">
+        <v>13</v>
+      </c>
+      <c r="L15">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12">
       <c r="A16">
         <v>2</v>
       </c>
       <c r="B16" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C16">
         <v>14.85</v>
       </c>
       <c r="D16">
-        <v>0.0</v>
+        <v>18.36</v>
       </c>
       <c r="E16">
-        <v>18.36</v>
+        <v>3.459038</v>
       </c>
       <c r="F16">
-        <v>3.459038</v>
+        <v>0.01106874</v>
       </c>
       <c r="G16">
-        <v>0.01106874</v>
+        <v>-1.0</v>
       </c>
       <c r="H16">
         <v>-1.0</v>
       </c>
       <c r="I16">
-        <v>-1.0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9">
+        <v>0.0</v>
+      </c>
+      <c r="J16">
+        <v>0.0</v>
+      </c>
+      <c r="K16" t="s">
+        <v>13</v>
+      </c>
+      <c r="L16">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12">
       <c r="A17">
         <v>2</v>
       </c>
       <c r="B17" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C17">
         <v>14.85</v>
       </c>
       <c r="D17">
-        <v>0.0</v>
+        <v>35.31</v>
       </c>
       <c r="E17">
-        <v>35.31</v>
+        <v>2.86671</v>
       </c>
       <c r="F17">
-        <v>2.86671</v>
+        <v>0.00772664</v>
       </c>
       <c r="G17">
-        <v>0.00772664</v>
+        <v>-1.0</v>
       </c>
       <c r="H17">
         <v>-1.0</v>
       </c>
       <c r="I17">
-        <v>-1.0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9">
+        <v>0.0</v>
+      </c>
+      <c r="J17">
+        <v>0.0</v>
+      </c>
+      <c r="K17" t="s">
+        <v>13</v>
+      </c>
+      <c r="L17">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12">
       <c r="A18">
         <v>2</v>
       </c>
       <c r="B18" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C18">
         <v>14.85</v>
       </c>
       <c r="D18">
-        <v>0.0</v>
+        <v>59.73</v>
       </c>
       <c r="E18">
-        <v>59.73</v>
+        <v>2.681798</v>
       </c>
       <c r="F18">
-        <v>2.681798</v>
+        <v>0.00610511</v>
       </c>
       <c r="G18">
-        <v>0.00610511</v>
+        <v>-1.0</v>
       </c>
       <c r="H18">
         <v>-1.0</v>
       </c>
       <c r="I18">
-        <v>-1.0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9">
+        <v>0.0</v>
+      </c>
+      <c r="J18">
+        <v>0.0</v>
+      </c>
+      <c r="K18" t="s">
+        <v>13</v>
+      </c>
+      <c r="L18">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12">
       <c r="A19">
         <v>2</v>
       </c>
       <c r="B19" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C19">
         <v>14.85</v>
       </c>
       <c r="D19">
-        <v>0.0</v>
+        <v>95.11</v>
       </c>
       <c r="E19">
-        <v>95.11</v>
+        <v>2.242077</v>
       </c>
       <c r="F19">
-        <v>2.242077</v>
+        <v>0.00512782</v>
       </c>
       <c r="G19">
-        <v>0.00512782</v>
+        <v>-1.0</v>
       </c>
       <c r="H19">
         <v>-1.0</v>
       </c>
       <c r="I19">
-        <v>-1.0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9">
+        <v>0.0</v>
+      </c>
+      <c r="J19">
+        <v>0.0</v>
+      </c>
+      <c r="K19" t="s">
+        <v>13</v>
+      </c>
+      <c r="L19">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12">
       <c r="A20">
         <v>2</v>
       </c>
       <c r="B20" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C20">
         <v>14.85</v>
       </c>
       <c r="D20">
-        <v>0.0</v>
+        <v>140.21</v>
       </c>
       <c r="E20">
-        <v>140.21</v>
+        <v>2.142624</v>
       </c>
       <c r="F20">
-        <v>2.142624</v>
+        <v>0.0045296</v>
       </c>
       <c r="G20">
-        <v>0.0045296</v>
+        <v>-1.0</v>
       </c>
       <c r="H20">
         <v>-1.0</v>
       </c>
       <c r="I20">
-        <v>-1.0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9">
+        <v>0.0</v>
+      </c>
+      <c r="J20">
+        <v>0.0</v>
+      </c>
+      <c r="K20" t="s">
+        <v>13</v>
+      </c>
+      <c r="L20">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12">
       <c r="A21">
         <v>2</v>
       </c>
       <c r="B21" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C21">
         <v>14.85</v>
       </c>
       <c r="D21">
-        <v>0.0</v>
+        <v>199.65</v>
       </c>
       <c r="E21">
-        <v>199.65</v>
+        <v>2.145291</v>
       </c>
       <c r="F21">
-        <v>2.145291</v>
+        <v>0.00410744</v>
       </c>
       <c r="G21">
-        <v>0.00410744</v>
+        <v>-1.0</v>
       </c>
       <c r="H21">
         <v>-1.0</v>
       </c>
       <c r="I21">
-        <v>-1.0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9">
+        <v>0.0</v>
+      </c>
+      <c r="J21">
+        <v>0.0</v>
+      </c>
+      <c r="K21" t="s">
+        <v>13</v>
+      </c>
+      <c r="L21">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12">
       <c r="A22">
         <v>2</v>
       </c>
       <c r="B22" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C22">
         <v>14.85</v>
       </c>
       <c r="D22">
-        <v>0.0</v>
+        <v>250.39</v>
       </c>
       <c r="E22">
-        <v>250.39</v>
+        <v>2.149538</v>
       </c>
       <c r="F22">
-        <v>2.149538</v>
+        <v>0.00388444</v>
       </c>
       <c r="G22">
-        <v>0.00388444</v>
+        <v>-1.0</v>
       </c>
       <c r="H22">
         <v>-1.0</v>
       </c>
       <c r="I22">
-        <v>-1.0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9">
+        <v>0.0</v>
+      </c>
+      <c r="J22">
+        <v>0.0</v>
+      </c>
+      <c r="K22" t="s">
+        <v>13</v>
+      </c>
+      <c r="L22">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12">
       <c r="A23">
         <v>2</v>
       </c>
       <c r="B23" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C23">
         <v>14.85</v>
       </c>
       <c r="D23">
-        <v>0.0</v>
+        <v>300.0</v>
       </c>
       <c r="E23">
-        <v>300.0</v>
+        <v>2.022008</v>
       </c>
       <c r="F23">
-        <v>2.022008</v>
+        <v>0.00372836</v>
       </c>
       <c r="G23">
-        <v>0.00372836</v>
+        <v>1.452357</v>
       </c>
       <c r="H23">
-        <v>1.452357</v>
+        <v>0.0150278</v>
       </c>
       <c r="I23">
-        <v>0.0150278</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9">
+        <v>0.0</v>
+      </c>
+      <c r="J23">
+        <v>0.0</v>
+      </c>
+      <c r="K23" t="s">
+        <v>13</v>
+      </c>
+      <c r="L23">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12">
       <c r="A24">
         <v>3</v>
       </c>
       <c r="B24" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C24">
         <v>17.85</v>
@@ -1090,404 +1309,530 @@
         <v>0.0</v>
       </c>
       <c r="E24">
-        <v>0.0</v>
+        <v>17.411771</v>
       </c>
       <c r="F24">
-        <v>17.411771</v>
+        <v>0.2916</v>
       </c>
       <c r="G24">
-        <v>0.2916</v>
+        <v>-1.0</v>
       </c>
       <c r="H24">
         <v>-1.0</v>
       </c>
       <c r="I24">
-        <v>-1.0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9">
+        <v>0.0</v>
+      </c>
+      <c r="J24">
+        <v>0.0</v>
+      </c>
+      <c r="K24" t="s">
+        <v>13</v>
+      </c>
+      <c r="L24">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12">
       <c r="A25">
         <v>3</v>
       </c>
       <c r="B25" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C25">
         <v>17.85</v>
       </c>
       <c r="D25">
-        <v>0.0</v>
+        <v>5.4</v>
       </c>
       <c r="E25">
-        <v>5.4</v>
+        <v>13.713733</v>
       </c>
       <c r="F25">
-        <v>13.713733</v>
+        <v>0.16490096</v>
       </c>
       <c r="G25">
-        <v>0.16490096</v>
+        <v>-1.0</v>
       </c>
       <c r="H25">
         <v>-1.0</v>
       </c>
       <c r="I25">
-        <v>-1.0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9">
+        <v>0.0</v>
+      </c>
+      <c r="J25">
+        <v>0.0</v>
+      </c>
+      <c r="K25" t="s">
+        <v>13</v>
+      </c>
+      <c r="L25">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12">
       <c r="A26">
         <v>3</v>
       </c>
       <c r="B26" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C26">
         <v>17.85</v>
       </c>
       <c r="D26">
-        <v>0.0</v>
+        <v>10.49</v>
       </c>
       <c r="E26">
-        <v>10.49</v>
+        <v>9.033066</v>
       </c>
       <c r="F26">
-        <v>9.033066</v>
+        <v>0.06996088</v>
       </c>
       <c r="G26">
-        <v>0.06996088</v>
+        <v>-1.0</v>
       </c>
       <c r="H26">
         <v>-1.0</v>
       </c>
       <c r="I26">
-        <v>-1.0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:9">
+        <v>0.0</v>
+      </c>
+      <c r="J26">
+        <v>0.0</v>
+      </c>
+      <c r="K26" t="s">
+        <v>13</v>
+      </c>
+      <c r="L26">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12">
       <c r="A27">
         <v>3</v>
       </c>
       <c r="B27" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C27">
         <v>17.85</v>
       </c>
       <c r="D27">
-        <v>0.0</v>
+        <v>14.94</v>
       </c>
       <c r="E27">
-        <v>14.94</v>
+        <v>7.210373</v>
       </c>
       <c r="F27">
-        <v>7.210373</v>
+        <v>0.04671906</v>
       </c>
       <c r="G27">
-        <v>0.04671906</v>
+        <v>-1.0</v>
       </c>
       <c r="H27">
         <v>-1.0</v>
       </c>
       <c r="I27">
-        <v>-1.0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:9">
+        <v>0.0</v>
+      </c>
+      <c r="J27">
+        <v>0.0</v>
+      </c>
+      <c r="K27" t="s">
+        <v>13</v>
+      </c>
+      <c r="L27">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12">
       <c r="A28">
         <v>3</v>
       </c>
       <c r="B28" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C28">
         <v>17.85</v>
       </c>
       <c r="D28">
-        <v>0.0</v>
+        <v>24.87</v>
       </c>
       <c r="E28">
-        <v>24.87</v>
+        <v>5.692268</v>
       </c>
       <c r="F28">
-        <v>5.692268</v>
+        <v>0.02884489</v>
       </c>
       <c r="G28">
-        <v>0.02884489</v>
+        <v>-1.0</v>
       </c>
       <c r="H28">
         <v>-1.0</v>
       </c>
       <c r="I28">
-        <v>-1.0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:9">
+        <v>0.0</v>
+      </c>
+      <c r="J28">
+        <v>0.0</v>
+      </c>
+      <c r="K28" t="s">
+        <v>13</v>
+      </c>
+      <c r="L28">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12">
       <c r="A29">
         <v>3</v>
       </c>
       <c r="B29" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C29">
         <v>17.85</v>
       </c>
       <c r="D29">
-        <v>0.0</v>
+        <v>40.04</v>
       </c>
       <c r="E29">
-        <v>40.04</v>
+        <v>4.793465</v>
       </c>
       <c r="F29">
-        <v>4.793465</v>
+        <v>0.0200434</v>
       </c>
       <c r="G29">
-        <v>0.0200434</v>
+        <v>-1.0</v>
       </c>
       <c r="H29">
         <v>-1.0</v>
       </c>
       <c r="I29">
-        <v>-1.0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9">
+        <v>0.0</v>
+      </c>
+      <c r="J29">
+        <v>0.0</v>
+      </c>
+      <c r="K29" t="s">
+        <v>13</v>
+      </c>
+      <c r="L29">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12">
       <c r="A30">
         <v>3</v>
       </c>
       <c r="B30" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C30">
         <v>17.85</v>
       </c>
       <c r="D30">
-        <v>0.0</v>
+        <v>60.41</v>
       </c>
       <c r="E30">
-        <v>60.41</v>
+        <v>4.191661</v>
       </c>
       <c r="F30">
-        <v>4.191661</v>
+        <v>0.01542391</v>
       </c>
       <c r="G30">
-        <v>0.01542391</v>
+        <v>-1.0</v>
       </c>
       <c r="H30">
         <v>-1.0</v>
       </c>
       <c r="I30">
-        <v>-1.0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:9">
+        <v>0.0</v>
+      </c>
+      <c r="J30">
+        <v>0.0</v>
+      </c>
+      <c r="K30" t="s">
+        <v>13</v>
+      </c>
+      <c r="L30">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12">
       <c r="A31">
         <v>3</v>
       </c>
       <c r="B31" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C31">
         <v>17.85</v>
       </c>
       <c r="D31">
-        <v>0.0</v>
+        <v>84.91</v>
       </c>
       <c r="E31">
-        <v>84.91</v>
+        <v>3.780834</v>
       </c>
       <c r="F31">
-        <v>3.780834</v>
+        <v>0.01279627</v>
       </c>
       <c r="G31">
-        <v>0.01279627</v>
+        <v>-1.0</v>
       </c>
       <c r="H31">
         <v>-1.0</v>
       </c>
       <c r="I31">
-        <v>-1.0</v>
-      </c>
-    </row>
-    <row r="32" spans="1:9">
+        <v>0.0</v>
+      </c>
+      <c r="J31">
+        <v>0.0</v>
+      </c>
+      <c r="K31" t="s">
+        <v>13</v>
+      </c>
+      <c r="L31">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12">
       <c r="A32">
         <v>3</v>
       </c>
       <c r="B32" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C32">
         <v>17.85</v>
       </c>
       <c r="D32">
-        <v>0.0</v>
+        <v>114.77</v>
       </c>
       <c r="E32">
-        <v>114.77</v>
+        <v>3.491126</v>
       </c>
       <c r="F32">
-        <v>3.491126</v>
+        <v>0.01106047</v>
       </c>
       <c r="G32">
-        <v>0.01106047</v>
+        <v>-1.0</v>
       </c>
       <c r="H32">
         <v>-1.0</v>
       </c>
       <c r="I32">
-        <v>-1.0</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9">
+        <v>0.0</v>
+      </c>
+      <c r="J32">
+        <v>0.0</v>
+      </c>
+      <c r="K32" t="s">
+        <v>13</v>
+      </c>
+      <c r="L32">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12">
       <c r="A33">
         <v>3</v>
       </c>
       <c r="B33" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C33">
         <v>17.85</v>
       </c>
       <c r="D33">
-        <v>0.0</v>
+        <v>149.79</v>
       </c>
       <c r="E33">
-        <v>149.79</v>
+        <v>3.323242</v>
       </c>
       <c r="F33">
-        <v>3.323242</v>
+        <v>0.00985622</v>
       </c>
       <c r="G33">
-        <v>0.00985622</v>
+        <v>-1.0</v>
       </c>
       <c r="H33">
         <v>-1.0</v>
       </c>
       <c r="I33">
-        <v>-1.0</v>
-      </c>
-    </row>
-    <row r="34" spans="1:9">
+        <v>0.0</v>
+      </c>
+      <c r="J33">
+        <v>0.0</v>
+      </c>
+      <c r="K33" t="s">
+        <v>13</v>
+      </c>
+      <c r="L33">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12">
       <c r="A34">
         <v>3</v>
       </c>
       <c r="B34" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C34">
         <v>17.85</v>
       </c>
       <c r="D34">
-        <v>0.0</v>
+        <v>190.14</v>
       </c>
       <c r="E34">
-        <v>190.14</v>
+        <v>3.288738</v>
       </c>
       <c r="F34">
-        <v>3.288738</v>
+        <v>0.00897658</v>
       </c>
       <c r="G34">
-        <v>0.00897658</v>
+        <v>-1.0</v>
       </c>
       <c r="H34">
         <v>-1.0</v>
       </c>
       <c r="I34">
-        <v>-1.0</v>
-      </c>
-    </row>
-    <row r="35" spans="1:9">
+        <v>0.0</v>
+      </c>
+      <c r="J34">
+        <v>0.0</v>
+      </c>
+      <c r="K34" t="s">
+        <v>13</v>
+      </c>
+      <c r="L34">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12">
       <c r="A35">
         <v>3</v>
       </c>
       <c r="B35" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C35">
         <v>17.85</v>
       </c>
       <c r="D35">
-        <v>0.0</v>
+        <v>235.03</v>
       </c>
       <c r="E35">
-        <v>235.03</v>
+        <v>3.209759</v>
       </c>
       <c r="F35">
-        <v>3.209759</v>
+        <v>0.00831996</v>
       </c>
       <c r="G35">
-        <v>0.00831996</v>
+        <v>-1.0</v>
       </c>
       <c r="H35">
         <v>-1.0</v>
       </c>
       <c r="I35">
-        <v>-1.0</v>
-      </c>
-    </row>
-    <row r="36" spans="1:9">
+        <v>0.0</v>
+      </c>
+      <c r="J35">
+        <v>0.0</v>
+      </c>
+      <c r="K35" t="s">
+        <v>13</v>
+      </c>
+      <c r="L35">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12">
       <c r="A36">
         <v>3</v>
       </c>
       <c r="B36" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C36">
         <v>17.85</v>
       </c>
       <c r="D36">
-        <v>0.0</v>
+        <v>280.26</v>
       </c>
       <c r="E36">
-        <v>280.26</v>
+        <v>2.823781</v>
       </c>
       <c r="F36">
-        <v>2.823781</v>
+        <v>0.00784831</v>
       </c>
       <c r="G36">
-        <v>0.00784831</v>
+        <v>-1.0</v>
       </c>
       <c r="H36">
         <v>-1.0</v>
       </c>
       <c r="I36">
-        <v>-1.0</v>
-      </c>
-    </row>
-    <row r="37" spans="1:9">
+        <v>0.0</v>
+      </c>
+      <c r="J36">
+        <v>0.0</v>
+      </c>
+      <c r="K36" t="s">
+        <v>13</v>
+      </c>
+      <c r="L36">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12">
       <c r="A37">
         <v>3</v>
       </c>
       <c r="B37" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C37">
         <v>17.85</v>
       </c>
       <c r="D37">
-        <v>0.0</v>
+        <v>305.0</v>
       </c>
       <c r="E37">
-        <v>305.0</v>
+        <v>2.928989</v>
       </c>
       <c r="F37">
-        <v>2.928989</v>
+        <v>0.00764224</v>
       </c>
       <c r="G37">
-        <v>0.00764224</v>
+        <v>2.52658</v>
       </c>
       <c r="H37">
-        <v>2.52658</v>
+        <v>0.03292264</v>
       </c>
       <c r="I37">
-        <v>0.03292264</v>
-      </c>
-    </row>
-    <row r="38" spans="1:9">
+        <v>0.0</v>
+      </c>
+      <c r="J37">
+        <v>0.0</v>
+      </c>
+      <c r="K37" t="s">
+        <v>13</v>
+      </c>
+      <c r="L37">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12">
       <c r="A38">
         <v>4</v>
       </c>
       <c r="B38" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C38">
         <v>20.85</v>
@@ -1496,259 +1841,340 @@
         <v>0.0</v>
       </c>
       <c r="E38">
-        <v>0.0</v>
+        <v>17.430589</v>
       </c>
       <c r="F38">
-        <v>17.430589</v>
+        <v>0.2601</v>
       </c>
       <c r="G38">
-        <v>0.2601</v>
+        <v>-1.0</v>
       </c>
       <c r="H38">
         <v>-1.0</v>
       </c>
       <c r="I38">
-        <v>-1.0</v>
-      </c>
-    </row>
-    <row r="39" spans="1:9">
+        <v>0.0</v>
+      </c>
+      <c r="J38">
+        <v>0.0</v>
+      </c>
+      <c r="K38" t="s">
+        <v>13</v>
+      </c>
+      <c r="L38">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12">
       <c r="A39">
         <v>4</v>
       </c>
       <c r="B39" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C39">
         <v>20.85</v>
       </c>
       <c r="D39">
-        <v>0.0</v>
+        <v>10.11</v>
       </c>
       <c r="E39">
-        <v>10.11</v>
+        <v>16.84467</v>
       </c>
       <c r="F39">
-        <v>16.84467</v>
+        <v>0.25619619</v>
       </c>
       <c r="G39">
-        <v>0.25619619</v>
+        <v>-1.0</v>
       </c>
       <c r="H39">
         <v>-1.0</v>
       </c>
       <c r="I39">
-        <v>-1.0</v>
-      </c>
-    </row>
-    <row r="40" spans="1:9">
+        <v>0.0</v>
+      </c>
+      <c r="J39">
+        <v>0.0</v>
+      </c>
+      <c r="K39" t="s">
+        <v>13</v>
+      </c>
+      <c r="L39">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12">
       <c r="A40">
         <v>4</v>
       </c>
       <c r="B40" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C40">
         <v>20.85</v>
       </c>
       <c r="D40">
-        <v>0.0</v>
+        <v>24.76</v>
       </c>
       <c r="E40">
-        <v>24.76</v>
+        <v>14.048812</v>
       </c>
       <c r="F40">
-        <v>14.048812</v>
+        <v>0.18446599</v>
       </c>
       <c r="G40">
-        <v>0.18446599</v>
+        <v>-1.0</v>
       </c>
       <c r="H40">
         <v>-1.0</v>
       </c>
       <c r="I40">
-        <v>-1.0</v>
-      </c>
-    </row>
-    <row r="41" spans="1:9">
+        <v>0.0</v>
+      </c>
+      <c r="J40">
+        <v>0.0</v>
+      </c>
+      <c r="K40" t="s">
+        <v>13</v>
+      </c>
+      <c r="L40">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12">
       <c r="A41">
         <v>4</v>
       </c>
       <c r="B41" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C41">
         <v>20.85</v>
       </c>
       <c r="D41">
-        <v>0.0</v>
+        <v>49.61</v>
       </c>
       <c r="E41">
-        <v>49.61</v>
+        <v>9.421758</v>
       </c>
       <c r="F41">
-        <v>9.421758</v>
+        <v>0.08318451</v>
       </c>
       <c r="G41">
-        <v>0.08318451</v>
+        <v>-1.0</v>
       </c>
       <c r="H41">
         <v>-1.0</v>
       </c>
       <c r="I41">
-        <v>-1.0</v>
-      </c>
-    </row>
-    <row r="42" spans="1:9">
+        <v>0.0</v>
+      </c>
+      <c r="J41">
+        <v>0.0</v>
+      </c>
+      <c r="K41" t="s">
+        <v>13</v>
+      </c>
+      <c r="L41">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12">
       <c r="A42">
         <v>4</v>
       </c>
       <c r="B42" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C42">
         <v>20.85</v>
       </c>
       <c r="D42">
-        <v>0.0</v>
+        <v>90.24</v>
       </c>
       <c r="E42">
-        <v>90.24</v>
+        <v>7.059156</v>
       </c>
       <c r="F42">
-        <v>7.059155</v>
+        <v>0.04465966</v>
       </c>
       <c r="G42">
-        <v>0.04465966</v>
+        <v>-1.0</v>
       </c>
       <c r="H42">
         <v>-1.0</v>
       </c>
       <c r="I42">
-        <v>-1.0</v>
-      </c>
-    </row>
-    <row r="43" spans="1:9">
+        <v>0.0</v>
+      </c>
+      <c r="J42">
+        <v>0.0</v>
+      </c>
+      <c r="K42" t="s">
+        <v>13</v>
+      </c>
+      <c r="L42">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="43" spans="1:12">
       <c r="A43">
         <v>4</v>
       </c>
       <c r="B43" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C43">
         <v>20.85</v>
       </c>
       <c r="D43">
-        <v>0.0</v>
+        <v>140.16</v>
       </c>
       <c r="E43">
-        <v>140.16</v>
+        <v>5.993199</v>
       </c>
       <c r="F43">
-        <v>5.993199</v>
+        <v>0.03127877</v>
       </c>
       <c r="G43">
-        <v>0.03127877</v>
+        <v>-1.0</v>
       </c>
       <c r="H43">
         <v>-1.0</v>
       </c>
       <c r="I43">
-        <v>-1.0</v>
-      </c>
-    </row>
-    <row r="44" spans="1:9">
+        <v>0.0</v>
+      </c>
+      <c r="J43">
+        <v>0.0</v>
+      </c>
+      <c r="K43" t="s">
+        <v>13</v>
+      </c>
+      <c r="L43">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="44" spans="1:12">
       <c r="A44">
         <v>4</v>
       </c>
       <c r="B44" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C44">
         <v>20.85</v>
       </c>
       <c r="D44">
-        <v>0.0</v>
+        <v>200.47</v>
       </c>
       <c r="E44">
-        <v>200.47</v>
+        <v>5.03884</v>
       </c>
       <c r="F44">
-        <v>5.03884</v>
+        <v>0.02464381</v>
       </c>
       <c r="G44">
-        <v>0.02464381</v>
+        <v>-1.0</v>
       </c>
       <c r="H44">
         <v>-1.0</v>
       </c>
       <c r="I44">
-        <v>-1.0</v>
-      </c>
-    </row>
-    <row r="45" spans="1:9">
+        <v>0.0</v>
+      </c>
+      <c r="J44">
+        <v>0.0</v>
+      </c>
+      <c r="K44" t="s">
+        <v>13</v>
+      </c>
+      <c r="L44">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="45" spans="1:12">
       <c r="A45">
         <v>4</v>
       </c>
       <c r="B45" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C45">
         <v>20.85</v>
       </c>
       <c r="D45">
-        <v>0.0</v>
+        <v>260.04</v>
       </c>
       <c r="E45">
-        <v>260.04</v>
+        <v>4.586802</v>
       </c>
       <c r="F45">
-        <v>4.586802</v>
+        <v>0.02121166</v>
       </c>
       <c r="G45">
-        <v>0.02121166</v>
+        <v>-1.0</v>
       </c>
       <c r="H45">
         <v>-1.0</v>
       </c>
       <c r="I45">
-        <v>-1.0</v>
-      </c>
-    </row>
-    <row r="46" spans="1:9">
+        <v>0.0</v>
+      </c>
+      <c r="J45">
+        <v>0.0</v>
+      </c>
+      <c r="K45" t="s">
+        <v>13</v>
+      </c>
+      <c r="L45">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="46" spans="1:12">
       <c r="A46">
         <v>4</v>
       </c>
       <c r="B46" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C46">
         <v>20.85</v>
       </c>
       <c r="D46">
-        <v>0.0</v>
+        <v>300.0</v>
       </c>
       <c r="E46">
-        <v>300.0</v>
+        <v>4.526651</v>
       </c>
       <c r="F46">
-        <v>4.526651</v>
+        <v>0.01967594</v>
       </c>
       <c r="G46">
-        <v>0.01967594</v>
+        <v>4.471779</v>
       </c>
       <c r="H46">
-        <v>4.471779</v>
+        <v>0.11321622</v>
       </c>
       <c r="I46">
-        <v>0.11321622</v>
-      </c>
-    </row>
-    <row r="47" spans="1:9">
+        <v>0.0</v>
+      </c>
+      <c r="J46">
+        <v>0.0</v>
+      </c>
+      <c r="K46" t="s">
+        <v>13</v>
+      </c>
+      <c r="L46">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="47" spans="1:12">
       <c r="A47">
         <v>5</v>
       </c>
       <c r="B47" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C47">
         <v>23.85</v>
@@ -1757,309 +2183,408 @@
         <v>0.0</v>
       </c>
       <c r="E47">
-        <v>0.0</v>
+        <v>14.694737</v>
       </c>
       <c r="F47">
-        <v>14.694737</v>
+        <v>0.2025</v>
       </c>
       <c r="G47">
-        <v>0.2025</v>
+        <v>-1.0</v>
       </c>
       <c r="H47">
         <v>-1.0</v>
       </c>
       <c r="I47">
-        <v>-1.0</v>
-      </c>
-    </row>
-    <row r="48" spans="1:9">
+        <v>0.0</v>
+      </c>
+      <c r="J47">
+        <v>0.0</v>
+      </c>
+      <c r="K47" t="s">
+        <v>13</v>
+      </c>
+      <c r="L47">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="48" spans="1:12">
       <c r="A48">
         <v>5</v>
       </c>
       <c r="B48" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C48">
         <v>23.85</v>
       </c>
       <c r="D48">
-        <v>0.0</v>
+        <v>5.94</v>
       </c>
       <c r="E48">
-        <v>5.94</v>
+        <v>15.088995</v>
       </c>
       <c r="F48">
-        <v>15.088995</v>
+        <v>0.2025</v>
       </c>
       <c r="G48">
-        <v>0.2025</v>
+        <v>-1.0</v>
       </c>
       <c r="H48">
         <v>-1.0</v>
       </c>
       <c r="I48">
-        <v>-1.0</v>
-      </c>
-    </row>
-    <row r="49" spans="1:9">
+        <v>0.0</v>
+      </c>
+      <c r="J48">
+        <v>0.0</v>
+      </c>
+      <c r="K48" t="s">
+        <v>13</v>
+      </c>
+      <c r="L48">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="49" spans="1:12">
       <c r="A49">
         <v>5</v>
       </c>
       <c r="B49" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C49">
         <v>23.85</v>
       </c>
       <c r="D49">
-        <v>0.0</v>
+        <v>14.22</v>
       </c>
       <c r="E49">
-        <v>14.22</v>
+        <v>15.91218</v>
       </c>
       <c r="F49">
-        <v>15.91218</v>
+        <v>0.20249991</v>
       </c>
       <c r="G49">
-        <v>0.20249991</v>
+        <v>-1.0</v>
       </c>
       <c r="H49">
         <v>-1.0</v>
       </c>
       <c r="I49">
-        <v>-1.0</v>
-      </c>
-    </row>
-    <row r="50" spans="1:9">
+        <v>0.0</v>
+      </c>
+      <c r="J49">
+        <v>0.0</v>
+      </c>
+      <c r="K49" t="s">
+        <v>13</v>
+      </c>
+      <c r="L49">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="50" spans="1:12">
       <c r="A50">
         <v>5</v>
       </c>
       <c r="B50" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C50">
         <v>23.85</v>
       </c>
       <c r="D50">
-        <v>0.0</v>
+        <v>27.86</v>
       </c>
       <c r="E50">
-        <v>27.86</v>
+        <v>15.239093</v>
       </c>
       <c r="F50">
-        <v>15.239093</v>
+        <v>0.20249867</v>
       </c>
       <c r="G50">
-        <v>0.20249867</v>
+        <v>-1.0</v>
       </c>
       <c r="H50">
         <v>-1.0</v>
       </c>
       <c r="I50">
-        <v>-1.0</v>
-      </c>
-    </row>
-    <row r="51" spans="1:9">
+        <v>0.0</v>
+      </c>
+      <c r="J50">
+        <v>0.0</v>
+      </c>
+      <c r="K50" t="s">
+        <v>13</v>
+      </c>
+      <c r="L50">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="51" spans="1:12">
       <c r="A51">
         <v>5</v>
       </c>
       <c r="B51" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C51">
         <v>23.85</v>
       </c>
       <c r="D51">
-        <v>0.0</v>
+        <v>50.45</v>
       </c>
       <c r="E51">
-        <v>50.45</v>
+        <v>15.545655</v>
       </c>
       <c r="F51">
-        <v>15.545655</v>
+        <v>0.20248574</v>
       </c>
       <c r="G51">
-        <v>0.20248574</v>
+        <v>-1.0</v>
       </c>
       <c r="H51">
         <v>-1.0</v>
       </c>
       <c r="I51">
-        <v>-1.0</v>
-      </c>
-    </row>
-    <row r="52" spans="1:9">
+        <v>0.0</v>
+      </c>
+      <c r="J51">
+        <v>0.0</v>
+      </c>
+      <c r="K51" t="s">
+        <v>13</v>
+      </c>
+      <c r="L51">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="52" spans="1:12">
       <c r="A52">
         <v>5</v>
       </c>
       <c r="B52" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C52">
         <v>23.85</v>
       </c>
       <c r="D52">
-        <v>0.0</v>
+        <v>80.05</v>
       </c>
       <c r="E52">
-        <v>80.05</v>
+        <v>15.517822</v>
       </c>
       <c r="F52">
-        <v>15.517822</v>
+        <v>0.20240969</v>
       </c>
       <c r="G52">
-        <v>0.20240969</v>
+        <v>-1.0</v>
       </c>
       <c r="H52">
         <v>-1.0</v>
       </c>
       <c r="I52">
-        <v>-1.0</v>
-      </c>
-    </row>
-    <row r="53" spans="1:9">
+        <v>0.0</v>
+      </c>
+      <c r="J52">
+        <v>0.0</v>
+      </c>
+      <c r="K52" t="s">
+        <v>13</v>
+      </c>
+      <c r="L52">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="53" spans="1:12">
       <c r="A53">
         <v>5</v>
       </c>
       <c r="B53" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C53">
         <v>23.85</v>
       </c>
       <c r="D53">
-        <v>0.0</v>
+        <v>120.15</v>
       </c>
       <c r="E53">
-        <v>120.15</v>
+        <v>15.300818</v>
       </c>
       <c r="F53">
-        <v>15.300818</v>
+        <v>0.20204332</v>
       </c>
       <c r="G53">
-        <v>0.20204332</v>
+        <v>-1.0</v>
       </c>
       <c r="H53">
         <v>-1.0</v>
       </c>
       <c r="I53">
-        <v>-1.0</v>
-      </c>
-    </row>
-    <row r="54" spans="1:9">
+        <v>0.0</v>
+      </c>
+      <c r="J53">
+        <v>0.0</v>
+      </c>
+      <c r="K53" t="s">
+        <v>13</v>
+      </c>
+      <c r="L53">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="54" spans="1:12">
       <c r="A54">
         <v>5</v>
       </c>
       <c r="B54" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C54">
         <v>23.85</v>
       </c>
       <c r="D54">
-        <v>0.0</v>
+        <v>164.66</v>
       </c>
       <c r="E54">
-        <v>164.66</v>
+        <v>15.512907</v>
       </c>
       <c r="F54">
-        <v>15.512907</v>
+        <v>0.2009071</v>
       </c>
       <c r="G54">
-        <v>0.2009071</v>
+        <v>-1.0</v>
       </c>
       <c r="H54">
         <v>-1.0</v>
       </c>
       <c r="I54">
-        <v>-1.0</v>
-      </c>
-    </row>
-    <row r="55" spans="1:9">
+        <v>0.0</v>
+      </c>
+      <c r="J54">
+        <v>0.0</v>
+      </c>
+      <c r="K54" t="s">
+        <v>13</v>
+      </c>
+      <c r="L54">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="55" spans="1:12">
       <c r="A55">
         <v>5</v>
       </c>
       <c r="B55" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C55">
         <v>23.85</v>
       </c>
       <c r="D55">
-        <v>0.0</v>
+        <v>215.22</v>
       </c>
       <c r="E55">
-        <v>215.22</v>
+        <v>15.234284</v>
       </c>
       <c r="F55">
-        <v>15.234284</v>
+        <v>0.19798525</v>
       </c>
       <c r="G55">
-        <v>0.19798525</v>
+        <v>-1.0</v>
       </c>
       <c r="H55">
         <v>-1.0</v>
       </c>
       <c r="I55">
-        <v>-1.0</v>
-      </c>
-    </row>
-    <row r="56" spans="1:9">
+        <v>0.0</v>
+      </c>
+      <c r="J55">
+        <v>0.0</v>
+      </c>
+      <c r="K55" t="s">
+        <v>13</v>
+      </c>
+      <c r="L55">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="56" spans="1:12">
       <c r="A56">
         <v>5</v>
       </c>
       <c r="B56" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C56">
         <v>23.85</v>
       </c>
       <c r="D56">
-        <v>0.0</v>
+        <v>265.45</v>
       </c>
       <c r="E56">
-        <v>265.45</v>
+        <v>13.859934</v>
       </c>
       <c r="F56">
-        <v>13.859934</v>
+        <v>0.1926158</v>
       </c>
       <c r="G56">
-        <v>0.1926158</v>
+        <v>-1.0</v>
       </c>
       <c r="H56">
         <v>-1.0</v>
       </c>
       <c r="I56">
-        <v>-1.0</v>
-      </c>
-    </row>
-    <row r="57" spans="1:9">
+        <v>0.0</v>
+      </c>
+      <c r="J56">
+        <v>0.0</v>
+      </c>
+      <c r="K56" t="s">
+        <v>13</v>
+      </c>
+      <c r="L56">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="57" spans="1:12">
       <c r="A57">
         <v>5</v>
       </c>
       <c r="B57" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C57">
         <v>23.85</v>
       </c>
       <c r="D57">
-        <v>0.0</v>
+        <v>305.0</v>
       </c>
       <c r="E57">
-        <v>305.0</v>
+        <v>14.74901</v>
       </c>
       <c r="F57">
-        <v>14.74901</v>
+        <v>0.18639072</v>
       </c>
       <c r="G57">
-        <v>0.18639072</v>
+        <v>8.814541</v>
       </c>
       <c r="H57">
-        <v>8.814541</v>
+        <v>0.53687406</v>
       </c>
       <c r="I57">
-        <v>0.53687406</v>
+        <v>0.0</v>
+      </c>
+      <c r="J57">
+        <v>0.0</v>
+      </c>
+      <c r="K57" t="s">
+        <v>13</v>
+      </c>
+      <c r="L57">
+        <v>1.25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>